<commit_message>
exp: continue to compute the results
</commit_message>
<xml_diff>
--- a/MLD01e_Results/Table42_AccuracyTable_Action_RiskReductionPast25_v1.xlsx
+++ b/MLD01e_Results/Table42_AccuracyTable_Action_RiskReductionPast25_v1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,28 +491,28 @@
         <v>42</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8115816767502161</v>
+        <v>0.8236819360414867</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7096774193548387</v>
+        <v>0.7288629737609329</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6703601108033241</v>
+        <v>0.6925207756232687</v>
       </c>
       <c r="G2" t="n">
-        <v>0.6894586894586895</v>
+        <v>0.7102272727272727</v>
       </c>
       <c r="H2" t="n">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="I2" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="J2" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="K2" t="n">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
@@ -526,28 +526,28 @@
         <v>42</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8055315471045809</v>
+        <v>0.8254105445116681</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6940509915014165</v>
+        <v>0.723463687150838</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6767955801104972</v>
+        <v>0.7154696132596685</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6853146853146853</v>
+        <v>0.7194444444444444</v>
       </c>
       <c r="H3" t="n">
-        <v>687</v>
+        <v>696</v>
       </c>
       <c r="I3" t="n">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="J3" t="n">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="K3" t="n">
-        <v>245</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4">
@@ -561,28 +561,28 @@
         <v>42</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8167675021607606</v>
+        <v>0.8349178910976663</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7286585365853658</v>
+        <v>0.7647058823529411</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6602209944751382</v>
+        <v>0.6823204419889503</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6927536231884058</v>
+        <v>0.7211678832116788</v>
       </c>
       <c r="H4" t="n">
-        <v>706</v>
+        <v>719</v>
       </c>
       <c r="I4" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="J4" t="n">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="K4" t="n">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5">
@@ -596,28 +596,28 @@
         <v>42</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8444252376836646</v>
+        <v>0.8409680207433017</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7527777777777778</v>
+        <v>0.7486033519553073</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7486187845303868</v>
+        <v>0.7403314917127072</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7506925207756233</v>
+        <v>0.7444444444444445</v>
       </c>
       <c r="H5" t="n">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="I5" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J5" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="K5" t="n">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6">
@@ -631,28 +631,28 @@
         <v>42</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8262748487467588</v>
+        <v>0.8418323249783924</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7476923076923077</v>
+        <v>0.7737003058103975</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6712707182320442</v>
+        <v>0.6988950276243094</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7074235807860262</v>
+        <v>0.7343976777939042</v>
       </c>
       <c r="H6" t="n">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="I6" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J6" t="n">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="K6" t="n">
-        <v>243</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7">
@@ -666,28 +666,28 @@
         <v>42</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8305963699222126</v>
+        <v>0.8392394122731202</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7331460674157303</v>
+        <v>0.7558139534883721</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7209944751381215</v>
+        <v>0.7182320441988951</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7270194986072424</v>
+        <v>0.7365439093484419</v>
       </c>
       <c r="H7" t="n">
-        <v>700</v>
+        <v>711</v>
       </c>
       <c r="I7" t="n">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="J7" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K7" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8">
@@ -701,28 +701,28 @@
         <v>42</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8055315471045809</v>
+        <v>0.8366464995678479</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6929577464788732</v>
+        <v>0.7436619718309859</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6795580110497238</v>
+        <v>0.7292817679558011</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6861924686192469</v>
+        <v>0.7364016736401674</v>
       </c>
       <c r="H8" t="n">
-        <v>686</v>
+        <v>704</v>
       </c>
       <c r="I8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="J8" t="n">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="K8" t="n">
-        <v>246</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9">
@@ -736,28 +736,28 @@
         <v>42</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8063958513396715</v>
+        <v>0.8297320656871219</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7053571428571429</v>
+        <v>0.7477477477477478</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6546961325966851</v>
+        <v>0.6878453038674033</v>
       </c>
       <c r="G9" t="n">
-        <v>0.6790830945558739</v>
+        <v>0.7165467625899281</v>
       </c>
       <c r="H9" t="n">
-        <v>696</v>
+        <v>711</v>
       </c>
       <c r="I9" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="J9" t="n">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="K9" t="n">
-        <v>237</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10">
@@ -771,28 +771,28 @@
         <v>42</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8166089965397924</v>
+        <v>0.8399653979238755</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7075208913649025</v>
+        <v>0.7417582417582418</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7036011080332411</v>
+        <v>0.7479224376731302</v>
       </c>
       <c r="G10" t="n">
-        <v>0.7055555555555556</v>
+        <v>0.7448275862068966</v>
       </c>
       <c r="H10" t="n">
-        <v>690</v>
+        <v>701</v>
       </c>
       <c r="I10" t="n">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="J10" t="n">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="K10" t="n">
-        <v>254</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11">
@@ -806,28 +806,28 @@
         <v>42</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8027681660899654</v>
+        <v>0.8382352941176471</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6873239436619718</v>
+        <v>0.7471590909090909</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6759002770083102</v>
+        <v>0.7285318559556787</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6815642458100558</v>
+        <v>0.7377279102384292</v>
       </c>
       <c r="H11" t="n">
-        <v>684</v>
+        <v>706</v>
       </c>
       <c r="I11" t="n">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="J11" t="n">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="K11" t="n">
-        <v>244</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12">
@@ -841,28 +841,28 @@
         <v>84</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8150388936905791</v>
+        <v>0.8305963699222126</v>
       </c>
       <c r="E12" t="n">
-        <v>0.723404255319149</v>
+        <v>0.746268656716418</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6592797783933518</v>
+        <v>0.6925207756232687</v>
       </c>
       <c r="G12" t="n">
-        <v>0.6898550724637681</v>
+        <v>0.7183908045977011</v>
       </c>
       <c r="H12" t="n">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="I12" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="J12" t="n">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="K12" t="n">
-        <v>238</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
@@ -876,28 +876,28 @@
         <v>84</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8141745894554884</v>
+        <v>0.8357821953327571</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7194029850746269</v>
+        <v>0.7457142857142857</v>
       </c>
       <c r="F13" t="n">
-        <v>0.6657458563535912</v>
+        <v>0.7209944751381215</v>
       </c>
       <c r="G13" t="n">
-        <v>0.6915351506456241</v>
+        <v>0.7331460674157303</v>
       </c>
       <c r="H13" t="n">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="I13" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="J13" t="n">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="K13" t="n">
-        <v>241</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14">
@@ -911,28 +911,28 @@
         <v>84</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8167675021607606</v>
+        <v>0.8357821953327571</v>
       </c>
       <c r="E14" t="n">
-        <v>0.7049180327868853</v>
+        <v>0.7275132275132276</v>
       </c>
       <c r="F14" t="n">
-        <v>0.7127071823204419</v>
+        <v>0.7596685082872928</v>
       </c>
       <c r="G14" t="n">
-        <v>0.7087912087912088</v>
+        <v>0.7432432432432432</v>
       </c>
       <c r="H14" t="n">
-        <v>687</v>
+        <v>692</v>
       </c>
       <c r="I14" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="J14" t="n">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="K14" t="n">
-        <v>258</v>
+        <v>275</v>
       </c>
     </row>
     <row r="15">
@@ -946,28 +946,28 @@
         <v>84</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8323249783923942</v>
+        <v>0.8504753673293</v>
       </c>
       <c r="E15" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.7632311977715878</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7292817679558011</v>
+        <v>0.7569060773480663</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7313019390581718</v>
+        <v>0.7600554785020804</v>
       </c>
       <c r="H15" t="n">
-        <v>699</v>
+        <v>710</v>
       </c>
       <c r="I15" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="J15" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="K15" t="n">
-        <v>264</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16">
@@ -981,28 +981,28 @@
         <v>84</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7934312878133103</v>
+        <v>0.8193604148660328</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6713091922005571</v>
+        <v>0.7217391304347827</v>
       </c>
       <c r="F16" t="n">
-        <v>0.6657458563535912</v>
+        <v>0.6878453038674033</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6685159500693482</v>
+        <v>0.7043847241867044</v>
       </c>
       <c r="H16" t="n">
-        <v>677</v>
+        <v>699</v>
       </c>
       <c r="I16" t="n">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="J16" t="n">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="K16" t="n">
-        <v>241</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17">
@@ -1016,28 +1016,28 @@
         <v>84</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8176318063958513</v>
+        <v>0.8323249783923942</v>
       </c>
       <c r="E17" t="n">
-        <v>0.7188405797101449</v>
+        <v>0.7441860465116279</v>
       </c>
       <c r="F17" t="n">
-        <v>0.6850828729281768</v>
+        <v>0.7071823204419889</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7015558698727016</v>
+        <v>0.7252124645892352</v>
       </c>
       <c r="H17" t="n">
-        <v>698</v>
+        <v>707</v>
       </c>
       <c r="I17" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="J17" t="n">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="K17" t="n">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18">
@@ -1051,28 +1051,28 @@
         <v>84</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8176318063958513</v>
+        <v>0.8409680207433017</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7175792507204611</v>
+        <v>0.7617647058823529</v>
       </c>
       <c r="F18" t="n">
-        <v>0.6878453038674033</v>
+        <v>0.7154696132596685</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7023977433004231</v>
+        <v>0.7378917378917379</v>
       </c>
       <c r="H18" t="n">
-        <v>697</v>
+        <v>714</v>
       </c>
       <c r="I18" t="n">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="J18" t="n">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="K18" t="n">
-        <v>249</v>
+        <v>259</v>
       </c>
     </row>
     <row r="19">
@@ -1086,28 +1086,28 @@
         <v>84</v>
       </c>
       <c r="D19" t="n">
-        <v>0.8228176318063959</v>
+        <v>0.8426966292134831</v>
       </c>
       <c r="E19" t="n">
-        <v>0.7315634218289085</v>
+        <v>0.7710843373493976</v>
       </c>
       <c r="F19" t="n">
-        <v>0.6850828729281768</v>
+        <v>0.7071823204419889</v>
       </c>
       <c r="G19" t="n">
-        <v>0.7075606276747504</v>
+        <v>0.7377521613832853</v>
       </c>
       <c r="H19" t="n">
-        <v>704</v>
+        <v>719</v>
       </c>
       <c r="I19" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="J19" t="n">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="K19" t="n">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="20">
@@ -1121,28 +1121,28 @@
         <v>84</v>
       </c>
       <c r="D20" t="n">
-        <v>0.8122837370242214</v>
+        <v>0.842560553633218</v>
       </c>
       <c r="E20" t="n">
-        <v>0.7130177514792899</v>
+        <v>0.7564469914040115</v>
       </c>
       <c r="F20" t="n">
-        <v>0.667590027700831</v>
+        <v>0.7313019390581718</v>
       </c>
       <c r="G20" t="n">
-        <v>0.6895565092989986</v>
+        <v>0.7436619718309859</v>
       </c>
       <c r="H20" t="n">
-        <v>698</v>
+        <v>710</v>
       </c>
       <c r="I20" t="n">
+        <v>85</v>
+      </c>
+      <c r="J20" t="n">
         <v>97</v>
       </c>
-      <c r="J20" t="n">
-        <v>120</v>
-      </c>
       <c r="K20" t="n">
-        <v>241</v>
+        <v>264</v>
       </c>
     </row>
     <row r="21">
@@ -1156,28 +1156,28 @@
         <v>84</v>
       </c>
       <c r="D21" t="n">
-        <v>0.8157439446366782</v>
+        <v>0.8321799307958477</v>
       </c>
       <c r="E21" t="n">
-        <v>0.7228915662650602</v>
+        <v>0.7448680351906158</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6648199445983379</v>
+        <v>0.7036011080332411</v>
       </c>
       <c r="G21" t="n">
-        <v>0.6926406926406926</v>
+        <v>0.7236467236467237</v>
       </c>
       <c r="H21" t="n">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="I21" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="J21" t="n">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="K21" t="n">
-        <v>240</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22">
@@ -1191,28 +1191,28 @@
         <v>126</v>
       </c>
       <c r="D22" t="n">
-        <v>0.8219533275713051</v>
+        <v>0.8392394122731202</v>
       </c>
       <c r="E22" t="n">
-        <v>0.7134986225895317</v>
+        <v>0.7521613832853026</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7174515235457064</v>
+        <v>0.7229916897506925</v>
       </c>
       <c r="G22" t="n">
-        <v>0.7154696132596685</v>
+        <v>0.7372881355932204</v>
       </c>
       <c r="H22" t="n">
-        <v>692</v>
+        <v>710</v>
       </c>
       <c r="I22" t="n">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="J22" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="K22" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23">
@@ -1226,28 +1226,28 @@
         <v>126</v>
       </c>
       <c r="D23" t="n">
-        <v>0.8029386343993086</v>
+        <v>0.8254105445116681</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6871508379888268</v>
+        <v>0.7285714285714285</v>
       </c>
       <c r="F23" t="n">
-        <v>0.6795580110497238</v>
+        <v>0.7044198895027625</v>
       </c>
       <c r="G23" t="n">
-        <v>0.6833333333333333</v>
+        <v>0.7162921348314607</v>
       </c>
       <c r="H23" t="n">
-        <v>683</v>
+        <v>700</v>
       </c>
       <c r="I23" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="J23" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="K23" t="n">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="24">
@@ -1261,28 +1261,28 @@
         <v>126</v>
       </c>
       <c r="D24" t="n">
-        <v>0.8245462402765773</v>
+        <v>0.8452895419187554</v>
       </c>
       <c r="E24" t="n">
-        <v>0.7264957264957265</v>
+        <v>0.754874651810585</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7044198895027625</v>
+        <v>0.7486187845303868</v>
       </c>
       <c r="G24" t="n">
-        <v>0.7152875175315568</v>
+        <v>0.7517337031900139</v>
       </c>
       <c r="H24" t="n">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="I24" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="J24" t="n">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="K24" t="n">
-        <v>255</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25">
@@ -1296,28 +1296,28 @@
         <v>126</v>
       </c>
       <c r="D25" t="n">
-        <v>0.8115816767502161</v>
+        <v>0.8280034572169404</v>
       </c>
       <c r="E25" t="n">
-        <v>0.7130177514792899</v>
+        <v>0.7418397626112759</v>
       </c>
       <c r="F25" t="n">
-        <v>0.6657458563535912</v>
+        <v>0.6906077348066298</v>
       </c>
       <c r="G25" t="n">
-        <v>0.6885714285714286</v>
+        <v>0.7153075822603719</v>
       </c>
       <c r="H25" t="n">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="I25" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="J25" t="n">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="K25" t="n">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26">
@@ -1331,28 +1331,28 @@
         <v>126</v>
       </c>
       <c r="D26" t="n">
-        <v>0.8228176318063959</v>
+        <v>0.8262748487467588</v>
       </c>
       <c r="E26" t="n">
-        <v>0.7150684931506849</v>
+        <v>0.721763085399449</v>
       </c>
       <c r="F26" t="n">
-        <v>0.7209944751381215</v>
+        <v>0.7237569060773481</v>
       </c>
       <c r="G26" t="n">
-        <v>0.7180192572214581</v>
+        <v>0.7227586206896551</v>
       </c>
       <c r="H26" t="n">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="I26" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="J26" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K26" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="27">
@@ -1366,16 +1366,16 @@
         <v>126</v>
       </c>
       <c r="D27" t="n">
-        <v>0.8236819360414867</v>
+        <v>0.8357821953327571</v>
       </c>
       <c r="E27" t="n">
-        <v>0.7219101123595506</v>
+        <v>0.7324324324324324</v>
       </c>
       <c r="F27" t="n">
-        <v>0.7099447513812155</v>
+        <v>0.7486187845303868</v>
       </c>
       <c r="G27" t="n">
-        <v>0.7158774373259053</v>
+        <v>0.7404371584699454</v>
       </c>
       <c r="H27" t="n">
         <v>696</v>
@@ -1384,10 +1384,10 @@
         <v>99</v>
       </c>
       <c r="J27" t="n">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="K27" t="n">
-        <v>257</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28">
@@ -1401,28 +1401,28 @@
         <v>126</v>
       </c>
       <c r="D28" t="n">
-        <v>0.8245462402765773</v>
+        <v>0.8375108038029386</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7401812688821753</v>
+        <v>0.7652439024390244</v>
       </c>
       <c r="F28" t="n">
-        <v>0.6767955801104972</v>
+        <v>0.6933701657458563</v>
       </c>
       <c r="G28" t="n">
-        <v>0.7070707070707071</v>
+        <v>0.7275362318840579</v>
       </c>
       <c r="H28" t="n">
-        <v>709</v>
+        <v>718</v>
       </c>
       <c r="I28" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="J28" t="n">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="K28" t="n">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="29">
@@ -1436,28 +1436,28 @@
         <v>126</v>
       </c>
       <c r="D29" t="n">
-        <v>0.8133102852203976</v>
+        <v>0.8349178910976663</v>
       </c>
       <c r="E29" t="n">
-        <v>0.7401315789473685</v>
+        <v>0.7647058823529411</v>
       </c>
       <c r="F29" t="n">
-        <v>0.6215469613259669</v>
+        <v>0.6823204419889503</v>
       </c>
       <c r="G29" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.7211678832116788</v>
       </c>
       <c r="H29" t="n">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="I29" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="J29" t="n">
-        <v>137</v>
+        <v>115</v>
       </c>
       <c r="K29" t="n">
-        <v>225</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30">
@@ -1471,28 +1471,28 @@
         <v>126</v>
       </c>
       <c r="D30" t="n">
-        <v>0.8148788927335641</v>
+        <v>0.8399653979238755</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7130434782608696</v>
+        <v>0.748587570621469</v>
       </c>
       <c r="F30" t="n">
-        <v>0.6814404432132964</v>
+        <v>0.7340720221606648</v>
       </c>
       <c r="G30" t="n">
-        <v>0.6968838526912181</v>
+        <v>0.7412587412587412</v>
       </c>
       <c r="H30" t="n">
-        <v>696</v>
+        <v>706</v>
       </c>
       <c r="I30" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="J30" t="n">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="K30" t="n">
-        <v>246</v>
+        <v>265</v>
       </c>
     </row>
     <row r="31">
@@ -1506,28 +1506,28 @@
         <v>126</v>
       </c>
       <c r="D31" t="n">
-        <v>0.8209342560553633</v>
+        <v>0.8477508650519031</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.7681159420289855</v>
       </c>
       <c r="F31" t="n">
-        <v>0.6703601108033241</v>
+        <v>0.7340720221606648</v>
       </c>
       <c r="G31" t="n">
-        <v>0.7004341534008683</v>
+        <v>0.7507082152974505</v>
       </c>
       <c r="H31" t="n">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="I31" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="J31" t="n">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="K31" t="n">
-        <v>242</v>
+        <v>265</v>
       </c>
     </row>
     <row r="32">
@@ -1541,28 +1541,28 @@
         <v>168</v>
       </c>
       <c r="D32" t="n">
-        <v>0.8089887640449438</v>
+        <v>0.8418323249783924</v>
       </c>
       <c r="E32" t="n">
-        <v>0.7046783625730995</v>
+        <v>0.7542857142857143</v>
       </c>
       <c r="F32" t="n">
-        <v>0.667590027700831</v>
+        <v>0.7313019390581718</v>
       </c>
       <c r="G32" t="n">
-        <v>0.6856330014224751</v>
+        <v>0.7426160337552743</v>
       </c>
       <c r="H32" t="n">
-        <v>695</v>
+        <v>710</v>
       </c>
       <c r="I32" t="n">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="J32" t="n">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="K32" t="n">
-        <v>241</v>
+        <v>264</v>
       </c>
     </row>
     <row r="33">
@@ -1576,28 +1576,28 @@
         <v>168</v>
       </c>
       <c r="D33" t="n">
-        <v>0.7934312878133103</v>
+        <v>0.8133102852203976</v>
       </c>
       <c r="E33" t="n">
-        <v>0.6782608695652174</v>
+        <v>0.7198795180722891</v>
       </c>
       <c r="F33" t="n">
-        <v>0.6464088397790055</v>
+        <v>0.6602209944751382</v>
       </c>
       <c r="G33" t="n">
-        <v>0.6619519094766619</v>
+        <v>0.6887608069164265</v>
       </c>
       <c r="H33" t="n">
-        <v>684</v>
+        <v>702</v>
       </c>
       <c r="I33" t="n">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="J33" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="K33" t="n">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="34">
@@ -1611,28 +1611,28 @@
         <v>168</v>
       </c>
       <c r="D34" t="n">
-        <v>0.8063958513396715</v>
+        <v>0.8176318063958513</v>
       </c>
       <c r="E34" t="n">
-        <v>0.6960227272727273</v>
+        <v>0.7091412742382271</v>
       </c>
       <c r="F34" t="n">
-        <v>0.6767955801104972</v>
+        <v>0.7071823204419889</v>
       </c>
       <c r="G34" t="n">
-        <v>0.6862745098039216</v>
+        <v>0.7081604426002767</v>
       </c>
       <c r="H34" t="n">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="I34" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J34" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="K34" t="n">
-        <v>245</v>
+        <v>256</v>
       </c>
     </row>
     <row r="35">
@@ -1646,28 +1646,28 @@
         <v>168</v>
       </c>
       <c r="D35" t="n">
-        <v>0.8133102852203976</v>
+        <v>0.8366464995678479</v>
       </c>
       <c r="E35" t="n">
-        <v>0.6983695652173914</v>
+        <v>0.7282321899736148</v>
       </c>
       <c r="F35" t="n">
-        <v>0.7099447513812155</v>
+        <v>0.7624309392265194</v>
       </c>
       <c r="G35" t="n">
-        <v>0.7041095890410959</v>
+        <v>0.7449392712550608</v>
       </c>
       <c r="H35" t="n">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="I35" t="n">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="J35" t="n">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="K35" t="n">
-        <v>257</v>
+        <v>276</v>
       </c>
     </row>
     <row r="36">
@@ -1681,28 +1681,28 @@
         <v>168</v>
       </c>
       <c r="D36" t="n">
-        <v>0.8210890233362144</v>
+        <v>0.8392394122731202</v>
       </c>
       <c r="E36" t="n">
-        <v>0.7476038338658147</v>
+        <v>0.7682926829268293</v>
       </c>
       <c r="F36" t="n">
-        <v>0.6464088397790055</v>
+        <v>0.6961325966850829</v>
       </c>
       <c r="G36" t="n">
-        <v>0.6933333333333334</v>
+        <v>0.7304347826086957</v>
       </c>
       <c r="H36" t="n">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="I36" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="J36" t="n">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="K36" t="n">
-        <v>234</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37">
@@ -1716,28 +1716,28 @@
         <v>168</v>
       </c>
       <c r="D37" t="n">
-        <v>0.8202247191011236</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="E37" t="n">
-        <v>0.71875</v>
+        <v>0.7628571428571429</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6988950276243094</v>
+        <v>0.7375690607734806</v>
       </c>
       <c r="G37" t="n">
-        <v>0.7086834733893558</v>
+        <v>0.75</v>
       </c>
       <c r="H37" t="n">
-        <v>696</v>
+        <v>712</v>
       </c>
       <c r="I37" t="n">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="J37" t="n">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="K37" t="n">
-        <v>253</v>
+        <v>267</v>
       </c>
     </row>
     <row r="38">
@@ -1751,28 +1751,28 @@
         <v>168</v>
       </c>
       <c r="D38" t="n">
-        <v>0.8418323249783924</v>
+        <v>0.8513396715643907</v>
       </c>
       <c r="E38" t="n">
-        <v>0.7896440129449838</v>
+        <v>0.8006329113924051</v>
       </c>
       <c r="F38" t="n">
-        <v>0.6740331491712708</v>
+        <v>0.6988950276243094</v>
       </c>
       <c r="G38" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.7463126843657817</v>
       </c>
       <c r="H38" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="I38" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J38" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="K38" t="n">
-        <v>244</v>
+        <v>253</v>
       </c>
     </row>
     <row r="39">
@@ -1786,28 +1786,28 @@
         <v>168</v>
       </c>
       <c r="D39" t="n">
-        <v>0.8133102852203976</v>
+        <v>0.8219533275713051</v>
       </c>
       <c r="E39" t="n">
-        <v>0.718562874251497</v>
+        <v>0.7307692307692307</v>
       </c>
       <c r="F39" t="n">
-        <v>0.6629834254143646</v>
+        <v>0.6823204419889503</v>
       </c>
       <c r="G39" t="n">
-        <v>0.6896551724137931</v>
+        <v>0.7057142857142857</v>
       </c>
       <c r="H39" t="n">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="I39" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J39" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="K39" t="n">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="40">
@@ -1821,28 +1821,28 @@
         <v>168</v>
       </c>
       <c r="D40" t="n">
-        <v>0.8365051903114187</v>
+        <v>0.856401384083045</v>
       </c>
       <c r="E40" t="n">
-        <v>0.75</v>
+        <v>0.7746478873239436</v>
       </c>
       <c r="F40" t="n">
-        <v>0.7146814404432132</v>
+        <v>0.7617728531855956</v>
       </c>
       <c r="G40" t="n">
-        <v>0.7319148936170212</v>
+        <v>0.7681564245810056</v>
       </c>
       <c r="H40" t="n">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="I40" t="n">
+        <v>80</v>
+      </c>
+      <c r="J40" t="n">
         <v>86</v>
       </c>
-      <c r="J40" t="n">
-        <v>103</v>
-      </c>
       <c r="K40" t="n">
-        <v>258</v>
+        <v>275</v>
       </c>
     </row>
     <row r="41">
@@ -1856,28 +1856,28 @@
         <v>168</v>
       </c>
       <c r="D41" t="n">
-        <v>0.8044982698961938</v>
+        <v>0.8235294117647058</v>
       </c>
       <c r="E41" t="n">
-        <v>0.6869806094182825</v>
+        <v>0.7198879551820728</v>
       </c>
       <c r="F41" t="n">
-        <v>0.6869806094182825</v>
+        <v>0.7119113573407202</v>
       </c>
       <c r="G41" t="n">
-        <v>0.6869806094182825</v>
+        <v>0.7158774373259053</v>
       </c>
       <c r="H41" t="n">
-        <v>682</v>
+        <v>695</v>
       </c>
       <c r="I41" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="J41" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="K41" t="n">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="42">
@@ -1891,28 +1891,28 @@
         <v>210</v>
       </c>
       <c r="D42" t="n">
-        <v>0.8167675021607606</v>
+        <v>0.8375108038029386</v>
       </c>
       <c r="E42" t="n">
-        <v>0.7159420289855073</v>
+        <v>0.7478510028653295</v>
       </c>
       <c r="F42" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.7229916897506925</v>
       </c>
       <c r="G42" t="n">
-        <v>0.6997167138810199</v>
+        <v>0.7352112676056338</v>
       </c>
       <c r="H42" t="n">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="I42" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="J42" t="n">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="K42" t="n">
-        <v>247</v>
+        <v>261</v>
       </c>
     </row>
     <row r="43">
@@ -1926,28 +1926,28 @@
         <v>210</v>
       </c>
       <c r="D43" t="n">
-        <v>0.8159031979256698</v>
+        <v>0.8409680207433017</v>
       </c>
       <c r="E43" t="n">
-        <v>0.7223880597014926</v>
+        <v>0.7587209302325582</v>
       </c>
       <c r="F43" t="n">
-        <v>0.6685082872928176</v>
+        <v>0.7209944751381215</v>
       </c>
       <c r="G43" t="n">
-        <v>0.6944045911047346</v>
+        <v>0.7393767705382436</v>
       </c>
       <c r="H43" t="n">
-        <v>702</v>
+        <v>712</v>
       </c>
       <c r="I43" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="J43" t="n">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="K43" t="n">
-        <v>242</v>
+        <v>261</v>
       </c>
     </row>
     <row r="44">
@@ -1961,28 +1961,28 @@
         <v>210</v>
       </c>
       <c r="D44" t="n">
-        <v>0.8254105445116681</v>
+        <v>0.8409680207433017</v>
       </c>
       <c r="E44" t="n">
-        <v>0.7366863905325444</v>
+        <v>0.7696969696969697</v>
       </c>
       <c r="F44" t="n">
-        <v>0.6878453038674033</v>
+        <v>0.7016574585635359</v>
       </c>
       <c r="G44" t="n">
-        <v>0.7114285714285714</v>
+        <v>0.7341040462427746</v>
       </c>
       <c r="H44" t="n">
-        <v>706</v>
+        <v>719</v>
       </c>
       <c r="I44" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="J44" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="K44" t="n">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="45">
@@ -1996,28 +1996,28 @@
         <v>210</v>
       </c>
       <c r="D45" t="n">
-        <v>0.8115816767502161</v>
+        <v>0.8418323249783924</v>
       </c>
       <c r="E45" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.7624633431085044</v>
       </c>
       <c r="F45" t="n">
-        <v>0.6629834254143646</v>
+        <v>0.7182320441988951</v>
       </c>
       <c r="G45" t="n">
-        <v>0.6876790830945558</v>
+        <v>0.7396870554765291</v>
       </c>
       <c r="H45" t="n">
-        <v>699</v>
+        <v>714</v>
       </c>
       <c r="I45" t="n">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="J45" t="n">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="K45" t="n">
-        <v>240</v>
+        <v>260</v>
       </c>
     </row>
     <row r="46">
@@ -2031,28 +2031,28 @@
         <v>210</v>
       </c>
       <c r="D46" t="n">
-        <v>0.8124459809853068</v>
+        <v>0.8340535868625756</v>
       </c>
       <c r="E46" t="n">
-        <v>0.7008310249307479</v>
+        <v>0.7401129943502824</v>
       </c>
       <c r="F46" t="n">
-        <v>0.6988950276243094</v>
+        <v>0.7237569060773481</v>
       </c>
       <c r="G46" t="n">
-        <v>0.6998616874135546</v>
+        <v>0.7318435754189944</v>
       </c>
       <c r="H46" t="n">
-        <v>687</v>
+        <v>703</v>
       </c>
       <c r="I46" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="J46" t="n">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="K46" t="n">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="47">
@@ -2066,28 +2066,28 @@
         <v>210</v>
       </c>
       <c r="D47" t="n">
-        <v>0.8107173725151253</v>
+        <v>0.8141745894554884</v>
       </c>
       <c r="E47" t="n">
-        <v>0.7109144542772862</v>
+        <v>0.7070422535211267</v>
       </c>
       <c r="F47" t="n">
-        <v>0.6657458563535912</v>
+        <v>0.6933701657458563</v>
       </c>
       <c r="G47" t="n">
-        <v>0.6875891583452212</v>
+        <v>0.7001394700139471</v>
       </c>
       <c r="H47" t="n">
-        <v>697</v>
+        <v>691</v>
       </c>
       <c r="I47" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="J47" t="n">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="K47" t="n">
-        <v>241</v>
+        <v>251</v>
       </c>
     </row>
     <row r="48">
@@ -2101,28 +2101,28 @@
         <v>210</v>
       </c>
       <c r="D48" t="n">
-        <v>0.8280034572169404</v>
+        <v>0.8383751080380294</v>
       </c>
       <c r="E48" t="n">
-        <v>0.7270194986072424</v>
+        <v>0.7450980392156863</v>
       </c>
       <c r="F48" t="n">
-        <v>0.7209944751381215</v>
+        <v>0.7348066298342542</v>
       </c>
       <c r="G48" t="n">
-        <v>0.723994452149792</v>
+        <v>0.7399165507649513</v>
       </c>
       <c r="H48" t="n">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="I48" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="J48" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="K48" t="n">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="49">
@@ -2136,28 +2136,28 @@
         <v>210</v>
       </c>
       <c r="D49" t="n">
-        <v>0.8089887640449438</v>
+        <v>0.8340535868625756</v>
       </c>
       <c r="E49" t="n">
-        <v>0.7067448680351907</v>
+        <v>0.7470930232558139</v>
       </c>
       <c r="F49" t="n">
-        <v>0.6657458563535912</v>
+        <v>0.7099447513812155</v>
       </c>
       <c r="G49" t="n">
-        <v>0.6856330014224751</v>
+        <v>0.7280453257790368</v>
       </c>
       <c r="H49" t="n">
-        <v>695</v>
+        <v>708</v>
       </c>
       <c r="I49" t="n">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="J49" t="n">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="K49" t="n">
-        <v>241</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50">
@@ -2171,28 +2171,28 @@
         <v>210</v>
       </c>
       <c r="D50" t="n">
-        <v>0.8148788927335641</v>
+        <v>0.8295847750865052</v>
       </c>
       <c r="E50" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.7265193370165746</v>
       </c>
       <c r="F50" t="n">
-        <v>0.6980609418282548</v>
+        <v>0.7285318559556787</v>
       </c>
       <c r="G50" t="n">
-        <v>0.7019498607242339</v>
+        <v>0.7275242047026279</v>
       </c>
       <c r="H50" t="n">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="I50" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="J50" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="K50" t="n">
-        <v>252</v>
+        <v>263</v>
       </c>
     </row>
     <row r="51">
@@ -2206,28 +2206,28 @@
         <v>210</v>
       </c>
       <c r="D51" t="n">
-        <v>0.8269896193771626</v>
+        <v>0.8416955017301038</v>
       </c>
       <c r="E51" t="n">
-        <v>0.7229916897506925</v>
+        <v>0.7572254335260116</v>
       </c>
       <c r="F51" t="n">
-        <v>0.7229916897506925</v>
+        <v>0.7257617728531855</v>
       </c>
       <c r="G51" t="n">
-        <v>0.7229916897506925</v>
+        <v>0.7411598302687411</v>
       </c>
       <c r="H51" t="n">
-        <v>695</v>
+        <v>711</v>
       </c>
       <c r="I51" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="J51" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K51" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="52">
@@ -2241,28 +2241,28 @@
         <v>252</v>
       </c>
       <c r="D52" t="n">
-        <v>0.8228176318063959</v>
+        <v>0.8444252376836646</v>
       </c>
       <c r="E52" t="n">
-        <v>0.7228571428571429</v>
+        <v>0.7520891364902507</v>
       </c>
       <c r="F52" t="n">
-        <v>0.7008310249307479</v>
+        <v>0.7479224376731302</v>
       </c>
       <c r="G52" t="n">
-        <v>0.7116736990154712</v>
+        <v>0.75</v>
       </c>
       <c r="H52" t="n">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="I52" t="n">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="J52" t="n">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="K52" t="n">
-        <v>253</v>
+        <v>270</v>
       </c>
     </row>
     <row r="53">
@@ -2276,28 +2276,28 @@
         <v>252</v>
       </c>
       <c r="D53" t="n">
-        <v>0.8193604148660328</v>
+        <v>0.8349178910976663</v>
       </c>
       <c r="E53" t="n">
-        <v>0.7119113573407202</v>
+        <v>0.7449856733524355</v>
       </c>
       <c r="F53" t="n">
-        <v>0.7099447513812155</v>
+        <v>0.7182320441988951</v>
       </c>
       <c r="G53" t="n">
-        <v>0.710926694329184</v>
+        <v>0.7313642756680732</v>
       </c>
       <c r="H53" t="n">
-        <v>691</v>
+        <v>706</v>
       </c>
       <c r="I53" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="J53" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="K53" t="n">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="54">
@@ -2311,28 +2311,28 @@
         <v>252</v>
       </c>
       <c r="D54" t="n">
-        <v>0.8176318063958513</v>
+        <v>0.8409680207433017</v>
       </c>
       <c r="E54" t="n">
-        <v>0.7138810198300283</v>
+        <v>0.7528409090909091</v>
       </c>
       <c r="F54" t="n">
-        <v>0.6961325966850829</v>
+        <v>0.7320441988950276</v>
       </c>
       <c r="G54" t="n">
-        <v>0.7048951048951049</v>
+        <v>0.742296918767507</v>
       </c>
       <c r="H54" t="n">
-        <v>694</v>
+        <v>708</v>
       </c>
       <c r="I54" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="J54" t="n">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="K54" t="n">
-        <v>252</v>
+        <v>265</v>
       </c>
     </row>
     <row r="55">
@@ -2346,28 +2346,28 @@
         <v>252</v>
       </c>
       <c r="D55" t="n">
-        <v>0.8193604148660328</v>
+        <v>0.8392394122731202</v>
       </c>
       <c r="E55" t="n">
-        <v>0.7283582089552239</v>
+        <v>0.7603550295857988</v>
       </c>
       <c r="F55" t="n">
-        <v>0.6740331491712708</v>
+        <v>0.7099447513812155</v>
       </c>
       <c r="G55" t="n">
-        <v>0.7001434720229556</v>
+        <v>0.7342857142857143</v>
       </c>
       <c r="H55" t="n">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="I55" t="n">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="J55" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="K55" t="n">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="56">
@@ -2381,28 +2381,28 @@
         <v>252</v>
       </c>
       <c r="D56" t="n">
-        <v>0.8228176318063959</v>
+        <v>0.8366464995678479</v>
       </c>
       <c r="E56" t="n">
-        <v>0.7357357357357357</v>
+        <v>0.7551622418879056</v>
       </c>
       <c r="F56" t="n">
-        <v>0.6767955801104972</v>
+        <v>0.7071823204419889</v>
       </c>
       <c r="G56" t="n">
-        <v>0.7050359712230215</v>
+        <v>0.7303851640513552</v>
       </c>
       <c r="H56" t="n">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="I56" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="J56" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="K56" t="n">
-        <v>245</v>
+        <v>256</v>
       </c>
     </row>
     <row r="57">
@@ -2416,28 +2416,28 @@
         <v>252</v>
       </c>
       <c r="D57" t="n">
-        <v>0.8133102852203976</v>
+        <v>0.8219533275713051</v>
       </c>
       <c r="E57" t="n">
-        <v>0.7109826589595376</v>
+        <v>0.7254335260115607</v>
       </c>
       <c r="F57" t="n">
-        <v>0.6795580110497238</v>
+        <v>0.6933701657458563</v>
       </c>
       <c r="G57" t="n">
-        <v>0.6949152542372882</v>
+        <v>0.7090395480225988</v>
       </c>
       <c r="H57" t="n">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="I57" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J57" t="n">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="K57" t="n">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="58">
@@ -2451,28 +2451,28 @@
         <v>252</v>
       </c>
       <c r="D58" t="n">
-        <v>0.808124459809853</v>
+        <v>0.8305963699222126</v>
       </c>
       <c r="E58" t="n">
-        <v>0.7108433734939759</v>
+        <v>0.7485029940119761</v>
       </c>
       <c r="F58" t="n">
-        <v>0.6519337016574586</v>
+        <v>0.6906077348066298</v>
       </c>
       <c r="G58" t="n">
-        <v>0.6801152737752162</v>
+        <v>0.7183908045977011</v>
       </c>
       <c r="H58" t="n">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="I58" t="n">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="J58" t="n">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K58" t="n">
-        <v>236</v>
+        <v>250</v>
       </c>
     </row>
     <row r="59">
@@ -2486,28 +2486,28 @@
         <v>252</v>
       </c>
       <c r="D59" t="n">
-        <v>0.8020743301642178</v>
+        <v>0.8202247191011236</v>
       </c>
       <c r="E59" t="n">
-        <v>0.6950146627565983</v>
+        <v>0.7291666666666666</v>
       </c>
       <c r="F59" t="n">
-        <v>0.6546961325966851</v>
+        <v>0.6767955801104972</v>
       </c>
       <c r="G59" t="n">
-        <v>0.6742532005689901</v>
+        <v>0.7020057306590258</v>
       </c>
       <c r="H59" t="n">
-        <v>691</v>
+        <v>704</v>
       </c>
       <c r="I59" t="n">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="J59" t="n">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="K59" t="n">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="60">
@@ -2521,22 +2521,22 @@
         <v>252</v>
       </c>
       <c r="D60" t="n">
-        <v>0.8451557093425606</v>
+        <v>0.8391003460207612</v>
       </c>
       <c r="E60" t="n">
-        <v>0.7630057803468208</v>
+        <v>0.7478753541076487</v>
       </c>
       <c r="F60" t="n">
         <v>0.7313019390581718</v>
       </c>
       <c r="G60" t="n">
-        <v>0.7468175388967468</v>
+        <v>0.7394957983193278</v>
       </c>
       <c r="H60" t="n">
-        <v>713</v>
+        <v>706</v>
       </c>
       <c r="I60" t="n">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="J60" t="n">
         <v>97</v>
@@ -2556,28 +2556,28 @@
         <v>252</v>
       </c>
       <c r="D61" t="n">
-        <v>0.8209342560553633</v>
+        <v>0.8373702422145328</v>
       </c>
       <c r="E61" t="n">
-        <v>0.72</v>
+        <v>0.7507246376811594</v>
       </c>
       <c r="F61" t="n">
-        <v>0.6980609418282548</v>
+        <v>0.7174515235457064</v>
       </c>
       <c r="G61" t="n">
-        <v>0.7088607594936709</v>
+        <v>0.7337110481586402</v>
       </c>
       <c r="H61" t="n">
-        <v>697</v>
+        <v>709</v>
       </c>
       <c r="I61" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="J61" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="K61" t="n">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="62">
@@ -2591,28 +2591,28 @@
         <v>294</v>
       </c>
       <c r="D62" t="n">
-        <v>0.8331892826274849</v>
+        <v>0.8513396715643907</v>
       </c>
       <c r="E62" t="n">
-        <v>0.7456140350877193</v>
+        <v>0.7661971830985915</v>
       </c>
       <c r="F62" t="n">
-        <v>0.7063711911357341</v>
+        <v>0.7534626038781164</v>
       </c>
       <c r="G62" t="n">
-        <v>0.7254623044096729</v>
+        <v>0.7597765363128491</v>
       </c>
       <c r="H62" t="n">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="I62" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="J62" t="n">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="K62" t="n">
-        <v>255</v>
+        <v>272</v>
       </c>
     </row>
     <row r="63">
@@ -2626,28 +2626,28 @@
         <v>294</v>
       </c>
       <c r="D63" t="n">
-        <v>0.8219533275713051</v>
+        <v>0.8444252376836646</v>
       </c>
       <c r="E63" t="n">
-        <v>0.7131147540983607</v>
+        <v>0.7645348837209303</v>
       </c>
       <c r="F63" t="n">
-        <v>0.7209944751381215</v>
+        <v>0.7265193370165746</v>
       </c>
       <c r="G63" t="n">
-        <v>0.717032967032967</v>
+        <v>0.7450424929178471</v>
       </c>
       <c r="H63" t="n">
-        <v>690</v>
+        <v>714</v>
       </c>
       <c r="I63" t="n">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="J63" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="K63" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="64">
@@ -2661,28 +2661,28 @@
         <v>294</v>
       </c>
       <c r="D64" t="n">
-        <v>0.8202247191011236</v>
+        <v>0.8366464995678479</v>
       </c>
       <c r="E64" t="n">
-        <v>0.7305389221556886</v>
+        <v>0.7521865889212828</v>
       </c>
       <c r="F64" t="n">
-        <v>0.6740331491712708</v>
+        <v>0.7127071823204419</v>
       </c>
       <c r="G64" t="n">
-        <v>0.7011494252873564</v>
+        <v>0.7319148936170212</v>
       </c>
       <c r="H64" t="n">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="I64" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J64" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="K64" t="n">
-        <v>244</v>
+        <v>258</v>
       </c>
     </row>
     <row r="65">
@@ -2696,28 +2696,28 @@
         <v>294</v>
       </c>
       <c r="D65" t="n">
-        <v>0.8098530682800346</v>
+        <v>0.8383751080380294</v>
       </c>
       <c r="E65" t="n">
-        <v>0.7017045454545454</v>
+        <v>0.7521613832853026</v>
       </c>
       <c r="F65" t="n">
-        <v>0.6823204419889503</v>
+        <v>0.7209944751381215</v>
       </c>
       <c r="G65" t="n">
-        <v>0.6918767507002801</v>
+        <v>0.7362482369534555</v>
       </c>
       <c r="H65" t="n">
-        <v>690</v>
+        <v>709</v>
       </c>
       <c r="I65" t="n">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="J65" t="n">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="K65" t="n">
-        <v>247</v>
+        <v>261</v>
       </c>
     </row>
     <row r="66">
@@ -2731,16 +2731,16 @@
         <v>294</v>
       </c>
       <c r="D66" t="n">
-        <v>0.8245462402765773</v>
+        <v>0.8305963699222126</v>
       </c>
       <c r="E66" t="n">
-        <v>0.729106628242075</v>
+        <v>0.7344632768361582</v>
       </c>
       <c r="F66" t="n">
-        <v>0.6988950276243094</v>
+        <v>0.7182320441988951</v>
       </c>
       <c r="G66" t="n">
-        <v>0.7136812411847673</v>
+        <v>0.7262569832402235</v>
       </c>
       <c r="H66" t="n">
         <v>701</v>
@@ -2749,10 +2749,10 @@
         <v>94</v>
       </c>
       <c r="J66" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="K66" t="n">
-        <v>253</v>
+        <v>260</v>
       </c>
     </row>
     <row r="67">
@@ -2766,28 +2766,28 @@
         <v>294</v>
       </c>
       <c r="D67" t="n">
-        <v>0.8184961106309421</v>
+        <v>0.8366464995678479</v>
       </c>
       <c r="E67" t="n">
-        <v>0.7196531791907514</v>
+        <v>0.7521865889212828</v>
       </c>
       <c r="F67" t="n">
-        <v>0.6878453038674033</v>
+        <v>0.7127071823204419</v>
       </c>
       <c r="G67" t="n">
-        <v>0.7033898305084746</v>
+        <v>0.7319148936170212</v>
       </c>
       <c r="H67" t="n">
-        <v>698</v>
+        <v>710</v>
       </c>
       <c r="I67" t="n">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="J67" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="K67" t="n">
-        <v>249</v>
+        <v>258</v>
       </c>
     </row>
     <row r="68">
@@ -2801,28 +2801,28 @@
         <v>294</v>
       </c>
       <c r="D68" t="n">
-        <v>0.8003457216940363</v>
+        <v>0.8297320656871219</v>
       </c>
       <c r="E68" t="n">
-        <v>0.6898550724637681</v>
+        <v>0.7363896848137536</v>
       </c>
       <c r="F68" t="n">
-        <v>0.6574585635359116</v>
+        <v>0.7099447513812155</v>
       </c>
       <c r="G68" t="n">
-        <v>0.6732673267326733</v>
+        <v>0.7229254571026723</v>
       </c>
       <c r="H68" t="n">
-        <v>688</v>
+        <v>703</v>
       </c>
       <c r="I68" t="n">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="J68" t="n">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="K68" t="n">
-        <v>238</v>
+        <v>257</v>
       </c>
     </row>
     <row r="69">
@@ -2836,28 +2836,28 @@
         <v>294</v>
       </c>
       <c r="D69" t="n">
-        <v>0.8107173725151253</v>
+        <v>0.8323249783923942</v>
       </c>
       <c r="E69" t="n">
-        <v>0.7002801120448179</v>
+        <v>0.7386363636363636</v>
       </c>
       <c r="F69" t="n">
-        <v>0.6906077348066298</v>
+        <v>0.7182320441988951</v>
       </c>
       <c r="G69" t="n">
-        <v>0.6954102920723226</v>
+        <v>0.7282913165266106</v>
       </c>
       <c r="H69" t="n">
-        <v>688</v>
+        <v>703</v>
       </c>
       <c r="I69" t="n">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="J69" t="n">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="K69" t="n">
-        <v>250</v>
+        <v>260</v>
       </c>
     </row>
     <row r="70">
@@ -2871,28 +2871,28 @@
         <v>294</v>
       </c>
       <c r="D70" t="n">
-        <v>0.8036332179930796</v>
+        <v>0.8209342560553633</v>
       </c>
       <c r="E70" t="n">
-        <v>0.6840659340659341</v>
+        <v>0.7175141242937854</v>
       </c>
       <c r="F70" t="n">
-        <v>0.6897506925207756</v>
+        <v>0.7036011080332411</v>
       </c>
       <c r="G70" t="n">
-        <v>0.6868965517241379</v>
+        <v>0.7104895104895105</v>
       </c>
       <c r="H70" t="n">
-        <v>680</v>
+        <v>695</v>
       </c>
       <c r="I70" t="n">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="J70" t="n">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="K70" t="n">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="71">
@@ -2906,28 +2906,28 @@
         <v>294</v>
       </c>
       <c r="D71" t="n">
-        <v>0.8183391003460208</v>
+        <v>0.842560553633218</v>
       </c>
       <c r="E71" t="n">
-        <v>0.7323076923076923</v>
+        <v>0.7753846153846153</v>
       </c>
       <c r="F71" t="n">
-        <v>0.6592797783933518</v>
+        <v>0.6980609418282548</v>
       </c>
       <c r="G71" t="n">
-        <v>0.6938775510204082</v>
+        <v>0.7346938775510204</v>
       </c>
       <c r="H71" t="n">
-        <v>708</v>
+        <v>722</v>
       </c>
       <c r="I71" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="J71" t="n">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="K71" t="n">
-        <v>238</v>
+        <v>252</v>
       </c>
     </row>
     <row r="72">
@@ -2941,28 +2941,28 @@
         <v>336</v>
       </c>
       <c r="D72" t="n">
-        <v>0.8141745894554884</v>
+        <v>0.8383751080380294</v>
       </c>
       <c r="E72" t="n">
-        <v>0.7050561797752809</v>
+        <v>0.7529069767441861</v>
       </c>
       <c r="F72" t="n">
-        <v>0.6952908587257618</v>
+        <v>0.7174515235457064</v>
       </c>
       <c r="G72" t="n">
-        <v>0.7001394700139471</v>
+        <v>0.7347517730496453</v>
       </c>
       <c r="H72" t="n">
-        <v>691</v>
+        <v>711</v>
       </c>
       <c r="I72" t="n">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="J72" t="n">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="K72" t="n">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="73">
@@ -2976,28 +2976,28 @@
         <v>336</v>
       </c>
       <c r="D73" t="n">
-        <v>0.8280034572169404</v>
+        <v>0.8470181503889369</v>
       </c>
       <c r="E73" t="n">
-        <v>0.7173333333333334</v>
+        <v>0.7479892761394102</v>
       </c>
       <c r="F73" t="n">
-        <v>0.7430939226519337</v>
+        <v>0.7707182320441989</v>
       </c>
       <c r="G73" t="n">
-        <v>0.7299864314789688</v>
+        <v>0.7591836734693878</v>
       </c>
       <c r="H73" t="n">
-        <v>689</v>
+        <v>701</v>
       </c>
       <c r="I73" t="n">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="J73" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="K73" t="n">
-        <v>269</v>
+        <v>279</v>
       </c>
     </row>
     <row r="74">
@@ -3011,28 +3011,28 @@
         <v>336</v>
       </c>
       <c r="D74" t="n">
-        <v>0.8046672428694901</v>
+        <v>0.8314606741573034</v>
       </c>
       <c r="E74" t="n">
-        <v>0.6988304093567251</v>
+        <v>0.7477744807121661</v>
       </c>
       <c r="F74" t="n">
-        <v>0.6602209944751382</v>
+        <v>0.6961325966850829</v>
       </c>
       <c r="G74" t="n">
-        <v>0.6789772727272727</v>
+        <v>0.721030042918455</v>
       </c>
       <c r="H74" t="n">
-        <v>692</v>
+        <v>710</v>
       </c>
       <c r="I74" t="n">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="J74" t="n">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="K74" t="n">
-        <v>239</v>
+        <v>252</v>
       </c>
     </row>
     <row r="75">
@@ -3046,28 +3046,28 @@
         <v>336</v>
       </c>
       <c r="D75" t="n">
-        <v>0.8262748487467588</v>
+        <v>0.8375108038029386</v>
       </c>
       <c r="E75" t="n">
-        <v>0.7388724035608308</v>
+        <v>0.757396449704142</v>
       </c>
       <c r="F75" t="n">
-        <v>0.6878453038674033</v>
+        <v>0.7071823204419889</v>
       </c>
       <c r="G75" t="n">
-        <v>0.7124463519313304</v>
+        <v>0.7314285714285714</v>
       </c>
       <c r="H75" t="n">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="I75" t="n">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="J75" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="K75" t="n">
-        <v>249</v>
+        <v>256</v>
       </c>
     </row>
     <row r="76">
@@ -3081,28 +3081,28 @@
         <v>336</v>
       </c>
       <c r="D76" t="n">
-        <v>0.8133102852203976</v>
+        <v>0.8280034572169404</v>
       </c>
       <c r="E76" t="n">
-        <v>0.7159763313609467</v>
+        <v>0.7308781869688386</v>
       </c>
       <c r="F76" t="n">
-        <v>0.6685082872928176</v>
+        <v>0.7127071823204419</v>
       </c>
       <c r="G76" t="n">
-        <v>0.6914285714285714</v>
+        <v>0.7216783216783217</v>
       </c>
       <c r="H76" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I76" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J76" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="K76" t="n">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="77">
@@ -3116,28 +3116,28 @@
         <v>336</v>
       </c>
       <c r="D77" t="n">
-        <v>0.8210890233362144</v>
+        <v>0.8444252376836646</v>
       </c>
       <c r="E77" t="n">
-        <v>0.7246376811594203</v>
+        <v>0.7676470588235295</v>
       </c>
       <c r="F77" t="n">
-        <v>0.6906077348066298</v>
+        <v>0.7209944751381215</v>
       </c>
       <c r="G77" t="n">
-        <v>0.7072135785007072</v>
+        <v>0.7435897435897436</v>
       </c>
       <c r="H77" t="n">
-        <v>700</v>
+        <v>716</v>
       </c>
       <c r="I77" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="J77" t="n">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="K77" t="n">
-        <v>250</v>
+        <v>261</v>
       </c>
     </row>
     <row r="78">
@@ -3151,28 +3151,28 @@
         <v>336</v>
       </c>
       <c r="D78" t="n">
-        <v>0.8072601555747623</v>
+        <v>0.8228176318063959</v>
       </c>
       <c r="E78" t="n">
-        <v>0.6991404011461319</v>
+        <v>0.7275362318840579</v>
       </c>
       <c r="F78" t="n">
-        <v>0.6740331491712708</v>
+        <v>0.6933701657458563</v>
       </c>
       <c r="G78" t="n">
-        <v>0.6863572433192686</v>
+        <v>0.71004243281471</v>
       </c>
       <c r="H78" t="n">
-        <v>690</v>
+        <v>701</v>
       </c>
       <c r="I78" t="n">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="J78" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="K78" t="n">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="79">
@@ -3186,28 +3186,28 @@
         <v>336</v>
       </c>
       <c r="D79" t="n">
-        <v>0.8107173725151253</v>
+        <v>0.8262748487467588</v>
       </c>
       <c r="E79" t="n">
-        <v>0.7025495750708215</v>
+        <v>0.7229916897506925</v>
       </c>
       <c r="F79" t="n">
-        <v>0.6850828729281768</v>
+        <v>0.7209944751381215</v>
       </c>
       <c r="G79" t="n">
-        <v>0.6937062937062937</v>
+        <v>0.7219917012448133</v>
       </c>
       <c r="H79" t="n">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="I79" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="J79" t="n">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="K79" t="n">
-        <v>248</v>
+        <v>261</v>
       </c>
     </row>
     <row r="80">
@@ -3221,28 +3221,28 @@
         <v>336</v>
       </c>
       <c r="D80" t="n">
-        <v>0.8304498269896193</v>
+        <v>0.8451557093425606</v>
       </c>
       <c r="E80" t="n">
-        <v>0.7586206896551724</v>
+        <v>0.7879746835443038</v>
       </c>
       <c r="F80" t="n">
-        <v>0.6703601108033241</v>
+        <v>0.6897506925207756</v>
       </c>
       <c r="G80" t="n">
-        <v>0.711764705882353</v>
+        <v>0.7355982274741507</v>
       </c>
       <c r="H80" t="n">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="I80" t="n">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J80" t="n">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="K80" t="n">
-        <v>242</v>
+        <v>249</v>
       </c>
     </row>
     <row r="81">
@@ -3256,28 +3256,28 @@
         <v>336</v>
       </c>
       <c r="D81" t="n">
-        <v>0.8096885813148789</v>
+        <v>0.8442906574394463</v>
       </c>
       <c r="E81" t="n">
-        <v>0.7104477611940299</v>
+        <v>0.7638483965014577</v>
       </c>
       <c r="F81" t="n">
-        <v>0.6592797783933518</v>
+        <v>0.7257617728531855</v>
       </c>
       <c r="G81" t="n">
-        <v>0.6839080459770115</v>
+        <v>0.7443181818181818</v>
       </c>
       <c r="H81" t="n">
-        <v>698</v>
+        <v>714</v>
       </c>
       <c r="I81" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="J81" t="n">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="K81" t="n">
-        <v>238</v>
+        <v>262</v>
       </c>
     </row>
     <row r="82">
@@ -3291,28 +3291,28 @@
         <v>378</v>
       </c>
       <c r="D82" t="n">
-        <v>0.8262748487467588</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="E82" t="n">
-        <v>0.7259887005649718</v>
+        <v>0.7534626038781164</v>
       </c>
       <c r="F82" t="n">
-        <v>0.7119113573407202</v>
+        <v>0.7534626038781164</v>
       </c>
       <c r="G82" t="n">
-        <v>0.7188811188811188</v>
+        <v>0.7534626038781164</v>
       </c>
       <c r="H82" t="n">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="I82" t="n">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="J82" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="K82" t="n">
-        <v>257</v>
+        <v>272</v>
       </c>
     </row>
     <row r="83">
@@ -3326,28 +3326,28 @@
         <v>378</v>
       </c>
       <c r="D83" t="n">
-        <v>0.8228176318063959</v>
+        <v>0.8210890233362144</v>
       </c>
       <c r="E83" t="n">
-        <v>0.7343283582089553</v>
+        <v>0.7220630372492837</v>
       </c>
       <c r="F83" t="n">
-        <v>0.6795580110497238</v>
+        <v>0.6961325966850829</v>
       </c>
       <c r="G83" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.7088607594936709</v>
       </c>
       <c r="H83" t="n">
-        <v>706</v>
+        <v>698</v>
       </c>
       <c r="I83" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="J83" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="K83" t="n">
-        <v>246</v>
+        <v>252</v>
       </c>
     </row>
     <row r="84">
@@ -3361,28 +3361,28 @@
         <v>378</v>
       </c>
       <c r="D84" t="n">
-        <v>0.8305963699222126</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="E84" t="n">
-        <v>0.7255434782608695</v>
+        <v>0.7473118279569892</v>
       </c>
       <c r="F84" t="n">
-        <v>0.7375690607734806</v>
+        <v>0.7679558011049724</v>
       </c>
       <c r="G84" t="n">
-        <v>0.7315068493150685</v>
+        <v>0.7574931880108992</v>
       </c>
       <c r="H84" t="n">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="I84" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="J84" t="n">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="K84" t="n">
-        <v>267</v>
+        <v>278</v>
       </c>
     </row>
     <row r="85">
@@ -3396,28 +3396,28 @@
         <v>378</v>
       </c>
       <c r="D85" t="n">
-        <v>0.8020743301642178</v>
+        <v>0.8236819360414867</v>
       </c>
       <c r="E85" t="n">
-        <v>0.6996996996996997</v>
+        <v>0.7453416149068323</v>
       </c>
       <c r="F85" t="n">
-        <v>0.643646408839779</v>
+        <v>0.6629834254143646</v>
       </c>
       <c r="G85" t="n">
-        <v>0.6705035971223021</v>
+        <v>0.7017543859649122</v>
       </c>
       <c r="H85" t="n">
-        <v>695</v>
+        <v>713</v>
       </c>
       <c r="I85" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="J85" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="K85" t="n">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="86">
@@ -3431,28 +3431,28 @@
         <v>378</v>
       </c>
       <c r="D86" t="n">
-        <v>0.8107173725151253</v>
+        <v>0.8210890233362144</v>
       </c>
       <c r="E86" t="n">
-        <v>0.7072463768115942</v>
+        <v>0.7259475218658892</v>
       </c>
       <c r="F86" t="n">
-        <v>0.6740331491712708</v>
+        <v>0.6878453038674033</v>
       </c>
       <c r="G86" t="n">
-        <v>0.6902404526166902</v>
+        <v>0.7063829787234043</v>
       </c>
       <c r="H86" t="n">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="I86" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="J86" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="K86" t="n">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="87">
@@ -3466,28 +3466,28 @@
         <v>378</v>
       </c>
       <c r="D87" t="n">
-        <v>0.8271391529818496</v>
+        <v>0.8349178910976663</v>
       </c>
       <c r="E87" t="n">
-        <v>0.7225274725274725</v>
+        <v>0.726790450928382</v>
       </c>
       <c r="F87" t="n">
-        <v>0.7265193370165746</v>
+        <v>0.7569060773480663</v>
       </c>
       <c r="G87" t="n">
-        <v>0.7245179063360881</v>
+        <v>0.7415426251691475</v>
       </c>
       <c r="H87" t="n">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="I87" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J87" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="K87" t="n">
-        <v>263</v>
+        <v>274</v>
       </c>
     </row>
     <row r="88">
@@ -3501,28 +3501,28 @@
         <v>378</v>
       </c>
       <c r="D88" t="n">
-        <v>0.8029386343993086</v>
+        <v>0.8262748487467588</v>
       </c>
       <c r="E88" t="n">
-        <v>0.6947674418604651</v>
+        <v>0.7360703812316716</v>
       </c>
       <c r="F88" t="n">
-        <v>0.6602209944751382</v>
+        <v>0.6933701657458563</v>
       </c>
       <c r="G88" t="n">
-        <v>0.6770538243626062</v>
+        <v>0.7140825035561877</v>
       </c>
       <c r="H88" t="n">
-        <v>690</v>
+        <v>705</v>
       </c>
       <c r="I88" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="J88" t="n">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="K88" t="n">
-        <v>239</v>
+        <v>251</v>
       </c>
     </row>
     <row r="89">
@@ -3536,28 +3536,28 @@
         <v>378</v>
       </c>
       <c r="D89" t="n">
-        <v>0.801210025929127</v>
+        <v>0.8305963699222126</v>
       </c>
       <c r="E89" t="n">
-        <v>0.6952662721893491</v>
+        <v>0.7455621301775148</v>
       </c>
       <c r="F89" t="n">
-        <v>0.649171270718232</v>
+        <v>0.6961325966850829</v>
       </c>
       <c r="G89" t="n">
-        <v>0.6714285714285714</v>
+        <v>0.72</v>
       </c>
       <c r="H89" t="n">
-        <v>692</v>
+        <v>709</v>
       </c>
       <c r="I89" t="n">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="J89" t="n">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="K89" t="n">
-        <v>235</v>
+        <v>252</v>
       </c>
     </row>
     <row r="90">
@@ -3571,28 +3571,28 @@
         <v>378</v>
       </c>
       <c r="D90" t="n">
-        <v>0.8200692041522492</v>
+        <v>0.8442906574394463</v>
       </c>
       <c r="E90" t="n">
-        <v>0.7243401759530792</v>
+        <v>0.7685459940652819</v>
       </c>
       <c r="F90" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.7174515235457064</v>
       </c>
       <c r="G90" t="n">
-        <v>0.7037037037037037</v>
+        <v>0.7421203438395415</v>
       </c>
       <c r="H90" t="n">
-        <v>701</v>
+        <v>717</v>
       </c>
       <c r="I90" t="n">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="J90" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="K90" t="n">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="91">
@@ -3606,28 +3606,28 @@
         <v>378</v>
       </c>
       <c r="D91" t="n">
-        <v>0.8131487889273357</v>
+        <v>0.846885813148789</v>
       </c>
       <c r="E91" t="n">
-        <v>0.7101449275362319</v>
+        <v>0.7754491017964071</v>
       </c>
       <c r="F91" t="n">
-        <v>0.6786703601108033</v>
+        <v>0.7174515235457064</v>
       </c>
       <c r="G91" t="n">
-        <v>0.6940509915014165</v>
+        <v>0.7453237410071942</v>
       </c>
       <c r="H91" t="n">
-        <v>695</v>
+        <v>720</v>
       </c>
       <c r="I91" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="J91" t="n">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="K91" t="n">
-        <v>245</v>
+        <v>259</v>
       </c>
     </row>
     <row r="92">
@@ -3641,28 +3641,28 @@
         <v>420</v>
       </c>
       <c r="D92" t="n">
-        <v>0.8141745894554884</v>
+        <v>0.8340535868625756</v>
       </c>
       <c r="E92" t="n">
-        <v>0.7212121212121212</v>
+        <v>0.7421203438395415</v>
       </c>
       <c r="F92" t="n">
-        <v>0.6592797783933518</v>
+        <v>0.7174515235457064</v>
       </c>
       <c r="G92" t="n">
-        <v>0.6888567293777135</v>
+        <v>0.7295774647887324</v>
       </c>
       <c r="H92" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="I92" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J92" t="n">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="K92" t="n">
-        <v>238</v>
+        <v>259</v>
       </c>
     </row>
     <row r="93">
@@ -3676,28 +3676,28 @@
         <v>420</v>
       </c>
       <c r="D93" t="n">
-        <v>0.8375108038029386</v>
+        <v>0.8496110630942092</v>
       </c>
       <c r="E93" t="n">
-        <v>0.7443820224719101</v>
+        <v>0.7568306010928961</v>
       </c>
       <c r="F93" t="n">
-        <v>0.7320441988950276</v>
+        <v>0.7651933701657458</v>
       </c>
       <c r="G93" t="n">
-        <v>0.7381615598885793</v>
+        <v>0.7609890109890109</v>
       </c>
       <c r="H93" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="I93" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J93" t="n">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="K93" t="n">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="94">
@@ -3711,28 +3711,28 @@
         <v>420</v>
       </c>
       <c r="D94" t="n">
-        <v>0.8141745894554884</v>
+        <v>0.8426966292134831</v>
       </c>
       <c r="E94" t="n">
-        <v>0.7118155619596542</v>
+        <v>0.7694610778443114</v>
       </c>
       <c r="F94" t="n">
-        <v>0.6823204419889503</v>
+        <v>0.7099447513812155</v>
       </c>
       <c r="G94" t="n">
-        <v>0.6967559943582511</v>
+        <v>0.7385057471264368</v>
       </c>
       <c r="H94" t="n">
-        <v>695</v>
+        <v>718</v>
       </c>
       <c r="I94" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="J94" t="n">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="K94" t="n">
-        <v>247</v>
+        <v>257</v>
       </c>
     </row>
     <row r="95">
@@ -3746,28 +3746,28 @@
         <v>420</v>
       </c>
       <c r="D95" t="n">
-        <v>0.8038029386343993</v>
+        <v>0.8219533275713051</v>
       </c>
       <c r="E95" t="n">
-        <v>0.6912181303116147</v>
+        <v>0.7178770949720671</v>
       </c>
       <c r="F95" t="n">
-        <v>0.6740331491712708</v>
+        <v>0.7099447513812155</v>
       </c>
       <c r="G95" t="n">
-        <v>0.6825174825174826</v>
+        <v>0.7138888888888889</v>
       </c>
       <c r="H95" t="n">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="I95" t="n">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="J95" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="K95" t="n">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="96">
@@ -3781,28 +3781,28 @@
         <v>420</v>
       </c>
       <c r="D96" t="n">
-        <v>0.8262748487467588</v>
+        <v>0.8513396715643907</v>
       </c>
       <c r="E96" t="n">
-        <v>0.7280453257790368</v>
+        <v>0.7653631284916201</v>
       </c>
       <c r="F96" t="n">
-        <v>0.7099447513812155</v>
+        <v>0.7569060773480663</v>
       </c>
       <c r="G96" t="n">
-        <v>0.7188811188811188</v>
+        <v>0.7611111111111111</v>
       </c>
       <c r="H96" t="n">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="I96" t="n">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="J96" t="n">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="K96" t="n">
-        <v>257</v>
+        <v>274</v>
       </c>
     </row>
     <row r="97">
@@ -3816,28 +3816,28 @@
         <v>420</v>
       </c>
       <c r="D97" t="n">
-        <v>0.8228176318063959</v>
+        <v>0.8280034572169404</v>
       </c>
       <c r="E97" t="n">
-        <v>0.7236467236467237</v>
+        <v>0.7308781869688386</v>
       </c>
       <c r="F97" t="n">
-        <v>0.7016574585635359</v>
+        <v>0.7127071823204419</v>
       </c>
       <c r="G97" t="n">
-        <v>0.7124824684431977</v>
+        <v>0.7216783216783217</v>
       </c>
       <c r="H97" t="n">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="I97" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="J97" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="K97" t="n">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="98">
@@ -3851,28 +3851,28 @@
         <v>420</v>
       </c>
       <c r="D98" t="n">
-        <v>0.8280034572169404</v>
+        <v>0.8305963699222126</v>
       </c>
       <c r="E98" t="n">
-        <v>0.7404129793510325</v>
+        <v>0.7357954545454546</v>
       </c>
       <c r="F98" t="n">
-        <v>0.6933701657458563</v>
+        <v>0.7154696132596685</v>
       </c>
       <c r="G98" t="n">
-        <v>0.7161198288159771</v>
+        <v>0.7254901960784313</v>
       </c>
       <c r="H98" t="n">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="I98" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="J98" t="n">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="K98" t="n">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="99">
@@ -3886,28 +3886,28 @@
         <v>420</v>
       </c>
       <c r="D99" t="n">
-        <v>0.8107173725151253</v>
+        <v>0.8314606741573034</v>
       </c>
       <c r="E99" t="n">
-        <v>0.7037037037037037</v>
+        <v>0.7406340057636888</v>
       </c>
       <c r="F99" t="n">
-        <v>0.6823204419889503</v>
+        <v>0.7099447513812155</v>
       </c>
       <c r="G99" t="n">
-        <v>0.6928471248246845</v>
+        <v>0.7249647390691114</v>
       </c>
       <c r="H99" t="n">
-        <v>691</v>
+        <v>705</v>
       </c>
       <c r="I99" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="J99" t="n">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="K99" t="n">
-        <v>247</v>
+        <v>257</v>
       </c>
     </row>
     <row r="100">
@@ -3921,28 +3921,28 @@
         <v>420</v>
       </c>
       <c r="D100" t="n">
-        <v>0.8261245674740484</v>
+        <v>0.8313148788927336</v>
       </c>
       <c r="E100" t="n">
-        <v>0.7409638554216867</v>
+        <v>0.7470238095238095</v>
       </c>
       <c r="F100" t="n">
-        <v>0.6814404432132964</v>
+        <v>0.6952908587257618</v>
       </c>
       <c r="G100" t="n">
-        <v>0.70995670995671</v>
+        <v>0.7202295552367288</v>
       </c>
       <c r="H100" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="I100" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J100" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="K100" t="n">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="101">
@@ -3956,28 +3956,28 @@
         <v>420</v>
       </c>
       <c r="D101" t="n">
-        <v>0.8148788927335641</v>
+        <v>0.8339100346020761</v>
       </c>
       <c r="E101" t="n">
-        <v>0.7247706422018348</v>
+        <v>0.7552870090634441</v>
       </c>
       <c r="F101" t="n">
-        <v>0.6565096952908587</v>
+        <v>0.6925207756232687</v>
       </c>
       <c r="G101" t="n">
-        <v>0.688953488372093</v>
+        <v>0.7225433526011561</v>
       </c>
       <c r="H101" t="n">
-        <v>705</v>
+        <v>714</v>
       </c>
       <c r="I101" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="J101" t="n">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="K101" t="n">
-        <v>237</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>